<commit_message>
feat: avance en creación de sql injection para pruebas de per testing
</commit_message>
<xml_diff>
--- a/src/test/resources/test-data.xlsx
+++ b/src/test/resources/test-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteban.canales\Desktop\Archivos\BackOffice\Proyectos ETL\Backend-ETL-Mercado-Spot\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8E56CDB-9508-4224-AC63-A089790D85EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49569A9E-C1D5-4920-8AA0-4E6EFF147B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Folio</t>
   </si>
@@ -67,6 +67,18 @@
   </si>
   <si>
     <t>Pagado</t>
+  </si>
+  <si>
+    <t>fechaEmision</t>
+  </si>
+  <si>
+    <t>fechaPago</t>
+  </si>
+  <si>
+    <t>tipoEntidad</t>
+  </si>
+  <si>
+    <t>DEUDOR</t>
   </si>
 </sst>
 </file>
@@ -112,13 +124,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,15 +412,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -435,8 +452,17 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -463,6 +489,15 @@
       </c>
       <c r="I2" t="s">
         <v>12</v>
+      </c>
+      <c r="J2" s="4">
+        <v>45292</v>
+      </c>
+      <c r="K2" s="4">
+        <v>45292</v>
+      </c>
+      <c r="L2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>